<commit_message>
Developer mapping: confirm 5 manual matches
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GZ6mf45gFCeDpGL3ireK6C
</commit_message>
<xml_diff>
--- a/docs/Bhoomija_Developer_Mapping.xlsx
+++ b/docs/Bhoomija_Developer_Mapping.xlsx
@@ -5517,33 +5517,37 @@
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>HOM-BSP-0007</t>
+          <t>JWL-NCK-0022-01</t>
         </is>
       </c>
       <c r="I88" s="3" t="inlineStr">
         <is>
-          <t>bawan-buti-bedspread-single</t>
+          <t>handcrafted-nagamese-necklace</t>
         </is>
       </c>
       <c r="J88" s="3" t="inlineStr">
         <is>
-          <t>52 Booti Single Bedspread (Teal Green base, Fruit motif)</t>
-        </is>
-      </c>
-      <c r="K88" s="3" t="inlineStr"/>
+          <t>Handcrafted Nagamese necklace</t>
+        </is>
+      </c>
+      <c r="K88" s="3" t="inlineStr">
+        <is>
+          <t>Azure (light) blue</t>
+        </is>
+      </c>
       <c r="L88" s="3" t="inlineStr">
         <is>
-          <t>DRAFT</t>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="M88" s="3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>High (confirmed)</t>
         </is>
       </c>
       <c r="N88" s="3" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496660054063</t>
+          <t>https://admin.shopify.com/store/bhoomija-2/products/8496643375151</t>
         </is>
       </c>
     </row>
@@ -5573,17 +5577,41 @@
       <c r="G89" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="H89" s="3" t="inlineStr"/>
-      <c r="I89" s="3" t="inlineStr"/>
-      <c r="J89" s="3" t="inlineStr"/>
-      <c r="K89" s="3" t="inlineStr"/>
-      <c r="L89" s="3" t="inlineStr"/>
-      <c r="M89" s="4" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
-      <c r="N89" s="3" t="inlineStr"/>
+      <c r="H89" s="3" t="inlineStr">
+        <is>
+          <t>JWL-NCK-0022-02</t>
+        </is>
+      </c>
+      <c r="I89" s="3" t="inlineStr">
+        <is>
+          <t>handcrafted-nagamese-necklace</t>
+        </is>
+      </c>
+      <c r="J89" s="3" t="inlineStr">
+        <is>
+          <t>Handcrafted Nagamese necklace</t>
+        </is>
+      </c>
+      <c r="K89" s="3" t="inlineStr">
+        <is>
+          <t>Cornflower (medium) blue</t>
+        </is>
+      </c>
+      <c r="L89" s="3" t="inlineStr">
+        <is>
+          <t>ACTIVE</t>
+        </is>
+      </c>
+      <c r="M89" s="3" t="inlineStr">
+        <is>
+          <t>High (confirmed)</t>
+        </is>
+      </c>
+      <c r="N89" s="3" t="inlineStr">
+        <is>
+          <t>https://admin.shopify.com/store/bhoomija-2/products/8496643375151</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="n">
@@ -7279,17 +7307,37 @@
       <c r="G118" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H118" s="3" t="inlineStr"/>
-      <c r="I118" s="3" t="inlineStr"/>
-      <c r="J118" s="3" t="inlineStr"/>
+      <c r="H118" s="3" t="inlineStr">
+        <is>
+          <t>JWL-NCK-0024</t>
+        </is>
+      </c>
+      <c r="I118" s="3" t="inlineStr">
+        <is>
+          <t>handcrafted-nagamese-necklace-1</t>
+        </is>
+      </c>
+      <c r="J118" s="3" t="inlineStr">
+        <is>
+          <t>Handcrafted Nagamese necklace - Green, Orange</t>
+        </is>
+      </c>
       <c r="K118" s="3" t="inlineStr"/>
-      <c r="L118" s="3" t="inlineStr"/>
-      <c r="M118" s="4" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
-      <c r="N118" s="3" t="inlineStr"/>
+      <c r="L118" s="3" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="M118" s="3" t="inlineStr">
+        <is>
+          <t>High (confirmed)</t>
+        </is>
+      </c>
+      <c r="N118" s="3" t="inlineStr">
+        <is>
+          <t>https://admin.shopify.com/store/bhoomija-2/products/8496643571759</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="3" t="n">
@@ -16292,17 +16340,37 @@
       <c r="G273" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="H273" s="3" t="inlineStr"/>
-      <c r="I273" s="3" t="inlineStr"/>
-      <c r="J273" s="3" t="inlineStr"/>
+      <c r="H273" s="3" t="inlineStr">
+        <is>
+          <t>HOM-CSC-0004</t>
+        </is>
+      </c>
+      <c r="I273" s="3" t="inlineStr">
+        <is>
+          <t>bawan-buti-cushion-cover</t>
+        </is>
+      </c>
+      <c r="J273" s="3" t="inlineStr">
+        <is>
+          <t>Bawan Buti cushion cover</t>
+        </is>
+      </c>
       <c r="K273" s="3" t="inlineStr"/>
-      <c r="L273" s="3" t="inlineStr"/>
-      <c r="M273" s="4" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
-      <c r="N273" s="3" t="inlineStr"/>
+      <c r="L273" s="3" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="M273" s="3" t="inlineStr">
+        <is>
+          <t>High (confirmed)</t>
+        </is>
+      </c>
+      <c r="N273" s="3" t="inlineStr">
+        <is>
+          <t>https://admin.shopify.com/store/bhoomija-2/products/8496659759151</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="3" t="n">
@@ -16852,17 +16920,37 @@
       <c r="G283" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="H283" s="3" t="inlineStr"/>
-      <c r="I283" s="3" t="inlineStr"/>
-      <c r="J283" s="3" t="inlineStr"/>
+      <c r="H283" s="3" t="inlineStr">
+        <is>
+          <t>HOM-BSP-0011</t>
+        </is>
+      </c>
+      <c r="I283" s="3" t="inlineStr">
+        <is>
+          <t>bawan-buti-bedspread-single-4</t>
+        </is>
+      </c>
+      <c r="J283" s="3" t="inlineStr">
+        <is>
+          <t>52 Booti Single Bedspread (Blue base, Santa Claus &amp; Snowman motif)</t>
+        </is>
+      </c>
       <c r="K283" s="3" t="inlineStr"/>
-      <c r="L283" s="3" t="inlineStr"/>
-      <c r="M283" s="4" t="inlineStr">
-        <is>
-          <t>Not found</t>
-        </is>
-      </c>
-      <c r="N283" s="3" t="inlineStr"/>
+      <c r="L283" s="3" t="inlineStr">
+        <is>
+          <t>DRAFT</t>
+        </is>
+      </c>
+      <c r="M283" s="3" t="inlineStr">
+        <is>
+          <t>High (confirmed)</t>
+        </is>
+      </c>
+      <c r="N283" s="3" t="inlineStr">
+        <is>
+          <t>https://admin.shopify.com/store/bhoomija-2/products/8496660283439</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="3" t="n">
@@ -18667,7 +18755,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -18841,54 +18929,54 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>JWL-NCK-0022-01</t>
+          <t>WEA-MKC-0003</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>handcrafted-nagamese-necklace</t>
+          <t>handwoven-mekhala-chador-from-assam-2</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Handcrafted Nagamese necklace</t>
+          <t>Handwoven Mekhala Chador from Assam</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Azure (light) blue</t>
+          <t>Default Title</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>DRAFT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496643375151</t>
+          <t>https://admin.shopify.com/store/bhoomija-2/products/8496646553647</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>JWL-NCK-0022-02</t>
+          <t>GHA-TRY-0001</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>handcrafted-nagamese-necklace</t>
+          <t>red-tikuli-hand-painted-tray</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Handcrafted Nagamese necklace</t>
+          <t>Red Tikuli hand painted tray</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Cornflower (medium) blue</t>
+          <t>Default Title</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -18898,24 +18986,24 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496643375151</t>
+          <t>https://admin.shopify.com/store/bhoomija-2/products/8496653140015</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>WEA-MKC-0003</t>
+          <t>HOM-CSC-0002</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>handwoven-mekhala-chador-from-assam-2</t>
+          <t>hand-embroidered-sujani-cushion-cover-16-by-16</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Handwoven Mekhala Chador from Assam</t>
+          <t>Hand embroidered Sujani cushion cover (16" by 16')</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -18930,61 +19018,61 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496646553647</t>
+          <t>https://admin.shopify.com/store/bhoomija-2/products/8496658186287</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GHA-TRY-0001</t>
+          <t>HOM-CSC-0005-BLUEWHITE</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>red-tikuli-hand-painted-tray</t>
+          <t>bawan-buti-cushion-cover-1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Red Tikuli hand painted tray</t>
+          <t>Bawan Buti cushion cover</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Default Title</t>
+          <t>Blue with White Elephant &amp; Leaf motif</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>ACTIVE</t>
+          <t>DRAFT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496653140015</t>
+          <t>https://admin.shopify.com/store/bhoomija-2/products/8496659791919</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>HOM-CSC-0002</t>
+          <t>HOM-CSC-0005-REDSTRIPED</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>hand-embroidered-sujani-cushion-cover-16-by-16</t>
+          <t>bawan-buti-cushion-cover-1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Hand embroidered Sujani cushion cover (16" by 16')</t>
+          <t>Bawan Buti cushion cover</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Default Title</t>
+          <t>Red striped with White Elephant motif</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -18994,14 +19082,14 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496658186287</t>
+          <t>https://admin.shopify.com/store/bhoomija-2/products/8496659791919</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>HOM-CSC-0005-BLUEWHITE</t>
+          <t>HOM-CSC-0005-REDWHITE</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -19016,7 +19104,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Blue with White Elephant &amp; Leaf motif</t>
+          <t>Red with White Nandi &amp; Fish motif</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -19033,7 +19121,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>HOM-CSC-0005-REDSTRIPED</t>
+          <t>HOM-CSC-0005-REDYELLOW</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -19048,7 +19136,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Red striped with White Elephant motif</t>
+          <t>Red with Yellow Nandi &amp; Fish motif</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -19065,7 +19153,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>HOM-CSC-0005-REDWHITE</t>
+          <t>HOM-CSC-0005-BLUENANDI</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -19080,7 +19168,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Red with White Nandi &amp; Fish motif</t>
+          <t>Blue with Nandi</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -19097,94 +19185,30 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>HOM-CSC-0005-REDYELLOW</t>
+          <t>WEA-MKW-0010</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>bawan-buti-cushion-cover-1</t>
+          <t>assamese-wrapper-1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Bawan Buti cushion cover</t>
+          <t>Assamese wrapper</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Red with Yellow Nandi &amp; Fish motif</t>
+          <t>Default Title</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>DRAFT</t>
+          <t>ACTIVE</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496659791919</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>HOM-CSC-0005-BLUENANDI</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>bawan-buti-cushion-cover-1</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Bawan Buti cushion cover</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Blue with Nandi</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>DRAFT</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>https://admin.shopify.com/store/bhoomija-2/products/8496659791919</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>WEA-MKW-0010</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>assamese-wrapper-1</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Assamese wrapper</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Default Title</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>ACTIVE</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
         <is>
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660512815</t>
         </is>

</xml_diff>

<commit_message>
Developer mapping: add live product links
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GZ6mf45gFCeDpGL3ireK6C
</commit_message>
<xml_diff>
--- a/docs/Bhoomija_Developer_Mapping.xlsx
+++ b/docs/Bhoomija_Developer_Mapping.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,6 +34,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF000000"/>
     </font>
   </fonts>
   <fills count="5">
@@ -71,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -82,6 +86,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -447,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N314"/>
+  <dimension ref="A1:O314"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -464,6 +469,7 @@
     <col width="9" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="50" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -537,6 +543,11 @@
           <t>Admin link</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Live product link</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
@@ -591,6 +602,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496633675823</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-jhola-bag</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -649,6 +665,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496633708591</t>
         </is>
       </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/teal-green-handwoven-cotton-moirang-phee-dupatta  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
@@ -711,6 +732,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496633806895</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-black-shapee-lanphee-stole  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -765,6 +791,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496633905199</t>
         </is>
       </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/cotton-silk-stole-with-hand-embroidered-turquoise-kantha-work  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -819,6 +850,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496633937967</t>
         </is>
       </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/reversible-pure-silk-hand-embroidered-kantha-stole  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -873,6 +909,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496633970735</t>
         </is>
       </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/peacock-blue-bishnupur-silk-dupatta-with-kantha-embroidery  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -927,6 +968,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496634069039</t>
         </is>
       </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/black-bishnupur-silk-dupatta-with-kantha-embroidery  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -981,6 +1027,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496635707439</t>
         </is>
       </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/natural-color-tussar-dupatta-with-hand-embroidered-kantha-work  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -1035,6 +1086,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496635805743</t>
         </is>
       </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/natural-color-tussar-dupatta-with-hand-embroidered-kantha-work-1  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
@@ -1089,6 +1145,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496635838511</t>
         </is>
       </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/slate-grey-kutch-work-dupatta-on-hand-woven-tussar  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
@@ -1143,6 +1204,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496636690479</t>
         </is>
       </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/salmon-pink-tussar-dupatta-with-hand-embroidered-kantha-work  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
@@ -1197,6 +1263,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496637345839</t>
         </is>
       </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/natural-color-tussar-dupatta-with-hand-embroidered-kantha-work-2  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -1251,6 +1322,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496637378607</t>
         </is>
       </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/blue-hand-emdroidered-cotton-dupatta-with-hand-embroidered-kantha-jaal-work  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
@@ -1305,6 +1381,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496637476911</t>
         </is>
       </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tree-of-life-kantha-hand-embroidered-bishnupur-silk-dress-material-2-5m  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
@@ -1363,6 +1444,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496637673519</t>
         </is>
       </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/contemporary-hand-painted-necklace-and-earring-set</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
@@ -1421,6 +1507,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496637739055</t>
         </is>
       </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/contemporary-hand-made-necklace-and-earring-set</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
@@ -1479,6 +1570,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496637804591</t>
         </is>
       </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madhubani-hand-painted-necklace-and-earring-set</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
@@ -1537,6 +1633,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496637870127</t>
         </is>
       </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/ajrakh-german-silver-necklace-and-earring-set</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -1595,6 +1696,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496637935663</t>
         </is>
       </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/ajrakh-german-silver-necklace-and-earring-set-1</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
@@ -1653,6 +1759,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496638001199</t>
         </is>
       </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-crafted-chess-board-patterned-necklace-and-earring-set</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
@@ -1711,6 +1822,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496639148079</t>
         </is>
       </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/macrame-hand-crafted-choker-set</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -1769,6 +1885,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496639246383</t>
         </is>
       </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-crafted-macrame-and-faux-pearl-nacklace-and-earring-set</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
@@ -1827,6 +1948,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496639279151</t>
         </is>
       </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-painted-and-hand-crafted-madhubani-necklace-and-earring-set</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
@@ -1885,6 +2011,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496639410223</t>
         </is>
       </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madhubani-hand-painted-necklace-and-earring-set-1</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
@@ -1943,6 +2074,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496639475759</t>
         </is>
       </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/fusion-dokra-and-jute-necklace-and-earrings-set</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
@@ -2001,6 +2137,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496639541295</t>
         </is>
       </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/brass-waterfall-necklace-and-earrings-set</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
@@ -2059,6 +2200,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496639639599</t>
         </is>
       </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/vintage-lahori-kantha-throw</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -2117,6 +2263,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496639672367</t>
         </is>
       </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/vintage-lahori-kantha-throw-1</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
@@ -2175,6 +2326,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496639737903</t>
         </is>
       </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/lord-shiv-maa-durga-with-their-children</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
@@ -2233,6 +2389,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496639803439</t>
         </is>
       </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/maa-durga-carried-by-devotee</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
@@ -2291,6 +2452,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496640032815</t>
         </is>
       </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/maa-lakshmi-on-her-owl</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
@@ -2349,6 +2515,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496640098351</t>
         </is>
       </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/mahishahur-mardini-with-maa-wearing-an-elaborate-crown</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
@@ -2407,6 +2578,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496640163887</t>
         </is>
       </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/maa-kali</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
@@ -2465,6 +2641,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496640262191</t>
         </is>
       </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madurkathi-mat</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
@@ -2523,6 +2704,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496640491567</t>
         </is>
       </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/maa-kali-1</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
@@ -2584,6 +2770,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496640589871</t>
         </is>
       </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bankura-horses</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
@@ -2642,6 +2833,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496640655407</t>
         </is>
       </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/durga-family-on-boat</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
@@ -2700,6 +2896,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496640720943</t>
         </is>
       </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/natural-tussar-color-tree-of-life-dupatta  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n">
@@ -2754,6 +2955,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496640852015</t>
         </is>
       </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/kantha-silk-dupatta  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n">
@@ -2808,6 +3014,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496640917551</t>
         </is>
       </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/cotton-silk-stole-with-black-hand-embroidered-kantha-work  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n">
@@ -2862,6 +3073,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496640983087</t>
         </is>
       </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-nakshi-kantha-on-handwoven-silk  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n">
@@ -2916,6 +3132,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496641114159</t>
         </is>
       </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-kantha-on-two-toned-handwoven-silk  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n">
@@ -2970,6 +3191,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496641212463</t>
         </is>
       </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/multi-strand-beads-necklace</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n">
@@ -3028,6 +3254,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496641245231</t>
         </is>
       </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/fusion-handcrafted-jute-necklace</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n">
@@ -3086,6 +3317,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496641310767</t>
         </is>
       </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/fusion-handembroidered-necklace</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n">
@@ -3144,6 +3380,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496641376303</t>
         </is>
       </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/macrame-multicolor-necklace</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
@@ -3203,6 +3444,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496641441839</t>
         </is>
       </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/traditional-kinnauri-pure-woollen-muffler</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n">
@@ -3262,6 +3508,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496641540143</t>
         </is>
       </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/mahishasur-mardini-22-by-30-madhubani-kachni-style  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n">
@@ -3321,6 +3572,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496641572911</t>
         </is>
       </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/maa-kali-22-by-30-bharni-style  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n">
@@ -3380,6 +3636,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496641736751</t>
         </is>
       </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/dashavtaar-11-by-30  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n">
@@ -3437,6 +3698,11 @@
       <c r="N52" s="3" t="inlineStr">
         <is>
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496641802287</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/ram-sita-vivah-11-5-by-30-5  (draft – not visible)</t>
         </is>
       </c>
     </row>
@@ -3610,6 +3876,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496641867823</t>
         </is>
       </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tripura-rangbatang-necklace</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n">
@@ -3664,6 +3935,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496641900591</t>
         </is>
       </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tripura-rangbatang-necklace-1</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n">
@@ -3718,6 +3994,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496641933359</t>
         </is>
       </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tripura-chandrahaar-long-necklace</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n">
@@ -3772,6 +4053,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496642129967</t>
         </is>
       </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tripura-chandrabaali-nabak-earrings</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n">
@@ -3826,6 +4112,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496642850863</t>
         </is>
       </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-long-coin-necklace-from-tripura</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n">
@@ -3880,6 +4171,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496642883631</t>
         </is>
       </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-long-coin-necklace-from-tripura-strung-with-red-beads</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="n">
@@ -3938,6 +4234,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643047471</t>
         </is>
       </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tripura-bagu</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n">
@@ -4000,6 +4301,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496618340399</t>
         </is>
       </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-handloom-pouch</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="n">
@@ -4062,6 +4368,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496618340399</t>
         </is>
       </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-handloom-pouch</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n">
@@ -4129,6 +4440,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496618340399</t>
         </is>
       </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-handloom-pouch</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n">
@@ -4191,6 +4507,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496618340399</t>
         </is>
       </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-handloom-pouch</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n">
@@ -4253,6 +4574,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496618340399</t>
         </is>
       </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-handloom-pouch</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="n">
@@ -4315,6 +4641,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496618340399</t>
         </is>
       </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-handloom-pouch</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="n">
@@ -4377,6 +4708,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496618340399</t>
         </is>
       </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-handloom-pouch</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="n">
@@ -4439,6 +4775,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496618504239</t>
         </is>
       </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-table-runner</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="n">
@@ -4506,6 +4847,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496618504239</t>
         </is>
       </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-table-runner</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n">
@@ -4568,6 +4914,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496618504239</t>
         </is>
       </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-table-runner</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="n">
@@ -4630,6 +4981,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496618504239</t>
         </is>
       </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-table-runner</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n">
@@ -4692,6 +5048,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496618504239</t>
         </is>
       </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-table-runner</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="n">
@@ -4754,6 +5115,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496618504239</t>
         </is>
       </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-table-runner</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n">
@@ -4816,6 +5182,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496618504239</t>
         </is>
       </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-table-runner</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="n">
@@ -4878,6 +5249,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496618504239</t>
         </is>
       </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-table-runner</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="n">
@@ -4940,6 +5316,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496618504239</t>
         </is>
       </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-table-runner</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="n">
@@ -4994,6 +5375,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496618602543</t>
         </is>
       </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/kauna-purse-white-flower-with-green-leaves  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n">
@@ -5048,6 +5434,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496618668079</t>
         </is>
       </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-kauna-u-bag  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="n">
@@ -5110,6 +5501,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643080239</t>
         </is>
       </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-handloom-coasters-set-of-6</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="n">
@@ -5177,6 +5573,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643080239</t>
         </is>
       </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-handloom-coasters-set-of-6</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="n">
@@ -5239,6 +5640,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643080239</t>
         </is>
       </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-handloom-coasters-set-of-6</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="n">
@@ -5301,6 +5707,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643080239</t>
         </is>
       </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-handloom-coasters-set-of-6</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="n">
@@ -5363,6 +5774,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643080239</t>
         </is>
       </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-handloom-coasters-set-of-6</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="n">
@@ -5425,6 +5841,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643080239</t>
         </is>
       </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-handloom-coasters-set-of-6</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="n">
@@ -5488,6 +5909,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643276847</t>
         </is>
       </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-belt-brown  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="n">
@@ -5550,6 +5976,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643375151</t>
         </is>
       </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="n">
@@ -5612,6 +6043,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643375151</t>
         </is>
       </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="n">
@@ -5668,6 +6104,11 @@
       <c r="N90" s="3" t="inlineStr">
         <is>
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643506223</t>
+        </is>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/nagamese-necklace-in-shades-of-yellow-green-with-bell-accent</t>
         </is>
       </c>
     </row>
@@ -5762,6 +6203,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643637295</t>
         </is>
       </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace-2</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="n">
@@ -5820,6 +6266,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643571759</t>
         </is>
       </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace-1  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="3" t="n">
@@ -5878,6 +6329,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643670063</t>
         </is>
       </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/nagamese-wrap</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="n">
@@ -5936,6 +6392,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643702831</t>
         </is>
       </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/mizo-wrapper-skirt</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="n">
@@ -5994,6 +6455,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643735599</t>
         </is>
       </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/assamese-mising-wrap-mekhla</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="n">
@@ -6056,6 +6522,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643768367</t>
         </is>
       </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-frame-with-wooden-stand</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="3" t="n">
@@ -6118,6 +6589,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643768367</t>
         </is>
       </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-frame-with-wooden-stand</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="n">
@@ -6180,6 +6656,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643768367</t>
         </is>
       </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-frame-with-wooden-stand</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="3" t="n">
@@ -6242,6 +6723,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643768367</t>
         </is>
       </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-frame-with-wooden-stand</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="n">
@@ -6304,6 +6790,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643768367</t>
         </is>
       </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-frame-with-wooden-stand</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="3" t="n">
@@ -6366,6 +6857,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643768367</t>
         </is>
       </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-frame-with-wooden-stand</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="n">
@@ -6428,6 +6924,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643768367</t>
         </is>
       </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-frame-with-wooden-stand</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="3" t="n">
@@ -6490,6 +6991,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643768367</t>
         </is>
       </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-frame-with-wooden-stand</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="n">
@@ -6552,6 +7058,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643768367</t>
         </is>
       </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-frame-with-wooden-stand</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="n">
@@ -6614,6 +7125,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643768367</t>
         </is>
       </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-frame-with-wooden-stand</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="3" t="n">
@@ -6676,6 +7192,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643768367</t>
         </is>
       </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-frame-with-wooden-stand</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="3" t="n">
@@ -6738,6 +7259,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643768367</t>
         </is>
       </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-frame-with-wooden-stand</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="n">
@@ -6800,6 +7326,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643997743</t>
         </is>
       </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/clutch-bag-made-with-hand-woven-assamese-silk  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="3" t="n">
@@ -6862,6 +7393,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643997743</t>
         </is>
       </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/clutch-bag-made-with-hand-woven-assamese-silk  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="n">
@@ -6924,6 +7460,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643997743</t>
         </is>
       </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/clutch-bag-made-with-hand-woven-assamese-silk  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="3" t="n">
@@ -6986,6 +7527,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643997743</t>
         </is>
       </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/clutch-bag-made-with-hand-woven-assamese-silk  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="3" t="n">
@@ -7048,6 +7594,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643997743</t>
         </is>
       </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/clutch-bag-made-with-hand-woven-assamese-silk  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="3" t="n">
@@ -7110,6 +7661,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643997743</t>
         </is>
       </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/clutch-bag-made-with-hand-woven-assamese-silk  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="3" t="n">
@@ -7172,6 +7728,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643997743</t>
         </is>
       </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/clutch-bag-made-with-hand-woven-assamese-silk  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="3" t="n">
@@ -7226,6 +7787,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496644128815</t>
         </is>
       </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace-4</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="3" t="n">
@@ -7280,6 +7846,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496644063279</t>
         </is>
       </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace-3</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="3" t="n">
@@ -7338,6 +7909,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496643571759</t>
         </is>
       </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace-1  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="3" t="n">
@@ -7397,6 +7973,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496645079087</t>
         </is>
       </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace-6</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="3" t="n">
@@ -7456,6 +8037,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496645701679</t>
         </is>
       </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace-7</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="3" t="n">
@@ -7515,6 +8101,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496645799983</t>
         </is>
       </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace-8</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="3" t="n">
@@ -7573,6 +8164,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496645865519</t>
         </is>
       </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace-9</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="3" t="n">
@@ -7631,6 +8227,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496644161583</t>
         </is>
       </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace-5  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="3" t="n">
@@ -7693,6 +8294,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496646062127</t>
         </is>
       </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace-10</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="3" t="n">
@@ -7755,6 +8361,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496646062127</t>
         </is>
       </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace-10</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="3" t="n">
@@ -7815,6 +8426,11 @@
       <c r="N126" s="3" t="inlineStr">
         <is>
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496646062127</t>
+        </is>
+      </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace-10</t>
         </is>
       </c>
     </row>
@@ -7914,6 +8530,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496646651951</t>
         </is>
       </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-mekhala-chador-from-assam-3  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="3" t="n">
@@ -7973,6 +8594,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496646225967</t>
         </is>
       </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-mekhala-chador-from-assam  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="3" t="n">
@@ -8031,6 +8657,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496646389807</t>
         </is>
       </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-mekhala-chador-from-assam-1  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="3" t="n">
@@ -8093,6 +8724,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496646946863</t>
         </is>
       </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sisters-of-the-north-east-clay-figurines</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="3" t="n">
@@ -8155,6 +8791,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496646946863</t>
         </is>
       </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sisters-of-the-north-east-clay-figurines</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="3" t="n">
@@ -8217,6 +8858,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496646946863</t>
         </is>
       </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sisters-of-the-north-east-clay-figurines</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="3" t="n">
@@ -8279,6 +8925,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496646946863</t>
         </is>
       </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sisters-of-the-north-east-clay-figurines</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="3" t="n">
@@ -8341,6 +8992,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496646946863</t>
         </is>
       </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sisters-of-the-north-east-clay-figurines</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="3" t="n">
@@ -8403,6 +9059,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496646946863</t>
         </is>
       </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sisters-of-the-north-east-clay-figurines</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="3" t="n">
@@ -8465,6 +9126,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496646946863</t>
         </is>
       </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sisters-of-the-north-east-clay-figurines</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="3" t="n">
@@ -8527,6 +9193,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496646946863</t>
         </is>
       </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sisters-of-the-north-east-clay-figurines</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="3" t="n">
@@ -8589,6 +9260,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496646946863</t>
         </is>
       </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sisters-of-the-north-east-clay-figurines</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="3" t="n">
@@ -8643,6 +9319,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496647012399</t>
         </is>
       </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/big-giraffe-planter-waterhyacinth</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="3" t="n">
@@ -8697,6 +9378,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496647045167</t>
         </is>
       </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/small-giraffe-planter-waterhyacinth</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="3" t="n">
@@ -8759,6 +9445,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496647077935</t>
         </is>
       </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/embroidered-moon-clutch-waterhyacinth  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="3" t="n">
@@ -8821,6 +9512,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496647077935</t>
         </is>
       </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/embroidered-moon-clutch-waterhyacinth  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="3" t="n">
@@ -8875,6 +9571,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496647143471</t>
         </is>
       </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/plain-moon-clutch-waterhyacinth  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="3" t="n">
@@ -8929,6 +9630,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496647176239</t>
         </is>
       </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/elephant-planter-waterhyacinth</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="3" t="n">
@@ -8983,6 +9689,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496647241775</t>
         </is>
       </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/water-hyacinth-handbag  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="3" t="n">
@@ -9037,6 +9748,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496647307311</t>
         </is>
       </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-water-hyacinth-bag  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="3" t="n">
@@ -9091,6 +9807,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496647372847</t>
         </is>
       </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace-11</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="3" t="n">
@@ -9145,6 +9866,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496647405615</t>
         </is>
       </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace-12</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="3" t="n">
@@ -9199,6 +9925,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496647471151</t>
         </is>
       </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace-13</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="3" t="n">
@@ -9253,6 +9984,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496647503919</t>
         </is>
       </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace-14</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="3" t="n">
@@ -9316,6 +10052,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496648618031</t>
         </is>
       </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace-15</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="3" t="n">
@@ -9370,6 +10111,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496648683567</t>
         </is>
       </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace-16</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="3" t="n">
@@ -9428,6 +10174,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496648716335</t>
         </is>
       </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handcrafted-nagamese-necklace-17</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="3" t="n">
@@ -9490,6 +10241,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496648814639</t>
         </is>
       </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-doli-bag-with-short-strap</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="3" t="n">
@@ -9552,6 +10308,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496648814639</t>
         </is>
       </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-doli-bag-with-short-strap</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="3" t="n">
@@ -9610,6 +10371,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649273391</t>
         </is>
       </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madurkathi-table-mat-set-including-runner-6-piece-set</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="3" t="n">
@@ -9668,6 +10434,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649306159</t>
         </is>
       </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madurkathi-table-mat-set-including-runner-6-piece-set-1</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="3" t="n">
@@ -9730,6 +10501,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649338927</t>
         </is>
       </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madurkathi-table-runner</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="3" t="n">
@@ -9792,6 +10568,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649338927</t>
         </is>
       </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madurkathi-table-runner</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="3" t="n">
@@ -9854,6 +10635,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649338927</t>
         </is>
       </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madurkathi-table-runner</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="3" t="n">
@@ -9916,6 +10702,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649338927</t>
         </is>
       </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madurkathi-table-runner</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="3" t="n">
@@ -9978,6 +10769,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649338927</t>
         </is>
       </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madurkathi-table-runner</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="3" t="n">
@@ -10040,6 +10836,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649371695</t>
         </is>
       </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/cushioned-madurkathi-yoga-mat</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="3" t="n">
@@ -10102,6 +10903,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649371695</t>
         </is>
       </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/cushioned-madurkathi-yoga-mat</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="3" t="n">
@@ -10164,6 +10970,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649371695</t>
         </is>
       </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/cushioned-madurkathi-yoga-mat</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="3" t="n">
@@ -10226,6 +11037,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649371695</t>
         </is>
       </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/cushioned-madurkathi-yoga-mat</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="3" t="n">
@@ -10288,6 +11104,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649437231</t>
         </is>
       </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/cushioned-madurkathi-ashon</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="3" t="n">
@@ -10350,6 +11171,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649437231</t>
         </is>
       </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/cushioned-madurkathi-ashon</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="3" t="n">
@@ -10412,6 +11238,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649437231</t>
         </is>
       </c>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/cushioned-madurkathi-ashon</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="3" t="n">
@@ -10474,6 +11305,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649437231</t>
         </is>
       </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/cushioned-madurkathi-ashon</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="3" t="n">
@@ -10532,6 +11368,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649469999</t>
         </is>
       </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madurkathi-table-runner-1</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="3" t="n">
@@ -10591,6 +11432,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649502767</t>
         </is>
       </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/durga-parivar-48-by-29  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="3" t="n">
@@ -10650,6 +11496,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649601071</t>
         </is>
       </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/raas-leela-24-by-29  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="3" t="n">
@@ -10709,6 +11560,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649633839</t>
         </is>
       </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/maa-kali-28-by-22  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="3" t="n">
@@ -10768,6 +11624,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649666607</t>
         </is>
       </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/mahishashur-mardini-maa-durga  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="3" t="n">
@@ -10827,6 +11688,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649699375</t>
         </is>
       </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/maa-saraswati-11-by-14  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="3" t="n">
@@ -10886,6 +11752,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649732143</t>
         </is>
       </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/maa-lakshmi-22-5-by-7  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="3" t="n">
@@ -10944,6 +11815,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649895983</t>
         </is>
       </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-maroon-jamdani-dupatta  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="3" t="n">
@@ -11007,6 +11883,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649764911</t>
         </is>
       </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-plum-cotton-jamdani-dupatta  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="3" t="n">
@@ -11065,6 +11946,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649830447</t>
         </is>
       </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-plum-cotton-jamdani-dupatta-1  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="3" t="n">
@@ -11123,6 +12009,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649928751</t>
         </is>
       </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-plum-teal-jamdani-dupatta  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="3" t="n">
@@ -11186,6 +12077,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649863215</t>
         </is>
       </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-teal-jamdani-dupatta  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="3" t="n">
@@ -11249,6 +12145,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496649994287</t>
         </is>
       </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-indigo-jamdani-dupatta  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="3" t="n">
@@ -11312,6 +12213,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496650059823</t>
         </is>
       </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-cotton-jamdani-dupatta  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="3" t="n">
@@ -11370,6 +12276,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496650092591</t>
         </is>
       </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-indigo-jamdani-dupatta-1  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="3" t="n">
@@ -11428,6 +12339,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496650125359</t>
         </is>
       </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/dhanekhali-stole  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="3" t="n">
@@ -11486,6 +12402,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496650190895</t>
         </is>
       </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/olive-handwoven-cotton-jamdani-stole  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="3" t="n">
@@ -11544,6 +12465,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496650354735</t>
         </is>
       </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-black-and-white-cotton-jamdani-stole  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="3" t="n">
@@ -11602,6 +12528,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496650453039</t>
         </is>
       </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-red-and-off-white-cotton-jamdani-stole  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="3" t="n">
@@ -11660,6 +12591,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496650518575</t>
         </is>
       </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/lilac-cotton-jamdani-stole  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="3" t="n">
@@ -11722,6 +12658,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496650584111</t>
         </is>
       </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-woven-cotton-silk-stole-with-extra-weft-motifs  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="3" t="n">
@@ -11784,6 +12725,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496650584111</t>
         </is>
       </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-woven-cotton-silk-stole-with-extra-weft-motifs  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="3" t="n">
@@ -11838,6 +12784,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496650846255</t>
         </is>
       </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-cotton-jamdani-stole-with-cute-tassels  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="3" t="n">
@@ -11896,6 +12847,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496650944559</t>
         </is>
       </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-cotton-dupatta-with-hand-embroidered-jamdani-motifs  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="3" t="n">
@@ -11950,6 +12906,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496650977327</t>
         </is>
       </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/red-handwoven-matka-silk-stole-with-zari-stripes  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="3" t="n">
@@ -12012,6 +12973,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496651010095</t>
         </is>
       </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/matka-silk-stole-with-jaquard-hand-woven-motifs  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="3" t="n">
@@ -12066,6 +13032,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496651075631</t>
         </is>
       </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/matka-silk-stole-with-extra-weft-motifs  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="3" t="n">
@@ -12128,6 +13099,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496651141167</t>
         </is>
       </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/matka-silk-shibori-dupatta  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="3" t="n">
@@ -12190,6 +13166,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496651141167</t>
         </is>
       </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/matka-silk-shibori-dupatta  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="3" t="n">
@@ -12244,6 +13225,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496651305007</t>
         </is>
       </c>
+      <c r="O201" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/matka-silk-dupatta-fulia-pink-with-blue-border  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="3" t="n">
@@ -12298,6 +13284,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496651403311</t>
         </is>
       </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/brown-linen-jamdani-dupatta  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="3" t="n">
@@ -12352,6 +13343,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496651436079</t>
         </is>
       </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/pink-linen-jamdani-stole  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="3" t="n">
@@ -12406,6 +13402,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496651501615</t>
         </is>
       </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/baluchari-unstitched-kurta-dupatta-set-magenta-on-off-white  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="3" t="n">
@@ -12469,6 +13470,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496651567151</t>
         </is>
       </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/jamdani-cotton-unstitched-kurta-dupatta-set-black  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="3" t="n">
@@ -12523,6 +13529,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496651665455</t>
         </is>
       </c>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/jamdani-cotton-unstitched-kurta-dupatta-set-taupe  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="3" t="n">
@@ -12577,6 +13588,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496651698223</t>
         </is>
       </c>
+      <c r="O207" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/corn-flower-blue-matka-baluchari-stole  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="3" t="n">
@@ -12639,6 +13655,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496651730991</t>
         </is>
       </c>
+      <c r="O208" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/silk-cotton-baluchari-dupatta  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="3" t="n">
@@ -12701,6 +13722,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496651730991</t>
         </is>
       </c>
+      <c r="O209" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/silk-cotton-baluchari-dupatta  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="3" t="n">
@@ -12759,6 +13785,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496651862063</t>
         </is>
       </c>
+      <c r="O210" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handmade-claycrafted-and-coloured-ek-chala-image-of-ma-durga-and-her-children</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="3" t="n">
@@ -12817,6 +13848,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496651894831</t>
         </is>
       </c>
+      <c r="O211" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handmade-claycrafted-and-copper-finished-ek-chala-image-of-ma-durga-and-her-children</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="3" t="n">
@@ -12873,6 +13909,11 @@
       <c r="N212" s="3" t="inlineStr">
         <is>
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496651927599</t>
+        </is>
+      </c>
+      <c r="O212" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handmade-claycrafted-image-of-rabindranath-tagore</t>
         </is>
       </c>
     </row>
@@ -12936,6 +13977,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496651960367</t>
         </is>
       </c>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sage-green-cylindrical-jamdani-lamp  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="3" t="n">
@@ -12995,6 +14041,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496652058671</t>
         </is>
       </c>
+      <c r="O214" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/red-square-jamdani-lamp</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="3" t="n">
@@ -13054,6 +14105,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496652288047</t>
         </is>
       </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/katha-table-lamp-with-wrought-iron-stand</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="3" t="n">
@@ -13113,6 +14169,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496653107247</t>
         </is>
       </c>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/cylindrical-gamosa-floor-lamp-red</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="3" t="n">
@@ -13167,6 +14228,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496653205551</t>
         </is>
       </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/black-tikuli-hand-painted-tray</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="3" t="n">
@@ -13221,6 +14287,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496653271087</t>
         </is>
       </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/black-tikuli-hand-painted-tray-1</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="3" t="n">
@@ -13275,6 +14346,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496653303855</t>
         </is>
       </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/red-tikuli-hand-painted-tray-1</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="3" t="n">
@@ -13329,6 +14405,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496653336623</t>
         </is>
       </c>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tikuli-handpainted-utility-box</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="3" t="n">
@@ -13383,6 +14464,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496653402159</t>
         </is>
       </c>
+      <c r="O221" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tikuli-handpainted-utility-box-1</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="3" t="n">
@@ -13437,6 +14523,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496653434927</t>
         </is>
       </c>
+      <c r="O222" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tikuli-handpainted-jewellery-box</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="3" t="n">
@@ -13495,6 +14586,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496653500463</t>
         </is>
       </c>
+      <c r="O223" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tikuli-handpainted-pen-stand</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="3" t="n">
@@ -13553,6 +14649,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496653533231</t>
         </is>
       </c>
+      <c r="O224" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tikuli-handpainted-tissue-holder</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="3" t="n">
@@ -13611,6 +14712,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496653598767</t>
         </is>
       </c>
+      <c r="O225" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tikuli-handpainted-tea-coaster-set-of-6</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="3" t="n">
@@ -13669,6 +14775,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496653697071</t>
         </is>
       </c>
+      <c r="O226" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tikuli-handpainted-tea-coaster-set-of-7</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="3" t="n">
@@ -13723,6 +14834,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496653729839</t>
         </is>
       </c>
+      <c r="O227" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tikuli-painting</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="3" t="n">
@@ -13785,6 +14901,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496653762607</t>
         </is>
       </c>
+      <c r="O228" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tikuli-painting-1</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="3" t="n">
@@ -13847,6 +14968,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496653762607</t>
         </is>
       </c>
+      <c r="O229" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tikuli-painting-1</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="3" t="n">
@@ -13909,6 +15035,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496653828143</t>
         </is>
       </c>
+      <c r="O230" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tikuli-hand-painted-mobile-stand  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="3" t="n">
@@ -13967,6 +15098,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496653893679</t>
         </is>
       </c>
+      <c r="O231" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tikuli-hand-painted-coasters-set-of-6</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="3" t="n">
@@ -14029,6 +15165,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496653926447</t>
         </is>
       </c>
+      <c r="O232" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madhubani-handpainted-clutch-bag  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="3" t="n">
@@ -14091,6 +15232,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496653926447</t>
         </is>
       </c>
+      <c r="O233" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madhubani-handpainted-clutch-bag  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="3" t="n">
@@ -14153,6 +15299,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496653926447</t>
         </is>
       </c>
+      <c r="O234" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madhubani-handpainted-clutch-bag  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="3" t="n">
@@ -14215,6 +15366,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496653991983</t>
         </is>
       </c>
+      <c r="O235" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madhubani-art-pouch  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="3" t="n">
@@ -14269,6 +15425,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496654057519</t>
         </is>
       </c>
+      <c r="O236" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madhubani-jute-thaila</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="3" t="n">
@@ -14332,6 +15493,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496654090287</t>
         </is>
       </c>
+      <c r="O237" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handpainted-madhubani-book-mark  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="3" t="n">
@@ -14390,6 +15556,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496654909487</t>
         </is>
       </c>
+      <c r="O238" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madhubani-slingbag  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="3" t="n">
@@ -14448,6 +15619,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496654942255</t>
         </is>
       </c>
+      <c r="O239" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tikuli-fridge-magnet  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="3" t="n">
@@ -14502,6 +15678,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496654975023</t>
         </is>
       </c>
+      <c r="O240" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tikuli-painting-without-frame</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="3" t="n">
@@ -14561,6 +15742,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496655007791</t>
         </is>
       </c>
+      <c r="O241" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hanuman-chalisa  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="3" t="n">
@@ -14619,6 +15805,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496655106095</t>
         </is>
       </c>
+      <c r="O242" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madhubani-painting-in-frame  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="3" t="n">
@@ -14677,6 +15868,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496655171631</t>
         </is>
       </c>
+      <c r="O243" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tikuli-paintings-in-frame  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="3" t="n">
@@ -14737,6 +15933,11 @@
       <c r="N244" s="3" t="inlineStr">
         <is>
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496655368239</t>
+        </is>
+      </c>
+      <c r="O244" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madhubani-clutch-purse  (draft – not visible)</t>
         </is>
       </c>
     </row>
@@ -14840,6 +16041,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496655368239</t>
         </is>
       </c>
+      <c r="O246" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madhubani-clutch-purse  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="3" t="n">
@@ -14898,6 +16104,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496655532079</t>
         </is>
       </c>
+      <c r="O247" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-sujani-stole-1  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="3" t="n">
@@ -14956,6 +16167,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496655466543</t>
         </is>
       </c>
+      <c r="O248" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-sujani-stole  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="3" t="n">
@@ -15014,6 +16230,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496655597615</t>
         </is>
       </c>
+      <c r="O249" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/intricately-hand-embroidered-silk-stole  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="3" t="n">
@@ -15072,6 +16293,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496655826991</t>
         </is>
       </c>
+      <c r="O250" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-sujani-cushion-cover-16by-16  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="3" t="n">
@@ -15130,6 +16356,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496655925295</t>
         </is>
       </c>
+      <c r="O251" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sujani-hand-embroidered-wall-hanging-unframed-prakriti</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="3" t="n">
@@ -15188,6 +16419,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496655990831</t>
         </is>
       </c>
+      <c r="O252" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sujani-hand-embroidered-wall-hanging-unframed-makhana-making</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" s="3" t="n">
@@ -15246,6 +16482,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496656056367</t>
         </is>
       </c>
+      <c r="O253" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sujani-hand-embroidered-wall-hanging-unframed-makhana-making-sujani-embroidery-in-process  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="3" t="n">
@@ -15308,6 +16549,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496656089135</t>
         </is>
       </c>
+      <c r="O254" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sujani-hand-embroidered-wall-hanging-unframed-sita-swayamvar  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="3" t="n">
@@ -15362,6 +16608,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496656121903</t>
         </is>
       </c>
+      <c r="O255" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/red-chanderi-hand-embroidered-sujani-dupatta  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="3" t="n">
@@ -15416,6 +16667,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496656220207</t>
         </is>
       </c>
+      <c r="O256" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/red-linen-hand-embroidered-sujani-dupatta  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="3" t="n">
@@ -15470,6 +16726,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496656252975</t>
         </is>
       </c>
+      <c r="O257" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/red-linen-hand-embroidered-sujani-dupatta-1  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="3" t="n">
@@ -15524,6 +16785,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496656285743</t>
         </is>
       </c>
+      <c r="O258" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/red-linen-hand-embroidered-sujani-dupatta-2  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="3" t="n">
@@ -15578,6 +16844,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496656351279</t>
         </is>
       </c>
+      <c r="O259" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/red-linen-hand-embroidered-sujani-dupatta-3  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="3" t="n">
@@ -15641,6 +16912,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496658120751</t>
         </is>
       </c>
+      <c r="O260" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/black-linen-hand-embroidered-sujani-dupatta  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="3" t="n">
@@ -15693,6 +16969,11 @@
       <c r="N261" s="3" t="inlineStr">
         <is>
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496658153519</t>
+        </is>
+      </c>
+      <c r="O261" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/yellow-bhagalpur-silk-hand-embroidered-sujani-dupatta  (draft – not visible)</t>
         </is>
       </c>
     </row>
@@ -15791,6 +17072,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496658219055</t>
         </is>
       </c>
+      <c r="O263" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-sujani-cushion-cover-14-by-14  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="3" t="n">
@@ -15849,6 +17135,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496658284591</t>
         </is>
       </c>
+      <c r="O264" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sujani-stole  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="3" t="n">
@@ -15907,6 +17198,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496659071023</t>
         </is>
       </c>
+      <c r="O265" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sujani-hand-embroidered-wall-hanging-unframedgrameen-a-village-scene  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="3" t="n">
@@ -15961,6 +17257,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496659595311</t>
         </is>
       </c>
+      <c r="O266" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tone-on-tone-handwoven-grey-tussar-stole-with-sujani-hand-embroidery  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="3" t="n">
@@ -16015,6 +17316,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496659628079</t>
         </is>
       </c>
+      <c r="O267" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-woven-pure-raw-silk-dupatta-with-ghicha-tussar-edges  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" s="3" t="n">
@@ -16069,6 +17375,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496659693615</t>
         </is>
       </c>
+      <c r="O268" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-woven-pure-raw-silk-dupatta-with-ghicha-tussar-edges-1  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="3" t="n">
@@ -16131,6 +17442,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496659726383</t>
         </is>
       </c>
+      <c r="O269" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cotton-jhola</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="3" t="n">
@@ -16193,6 +17509,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496659726383</t>
         </is>
       </c>
+      <c r="O270" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cotton-jhola</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="3" t="n">
@@ -16255,6 +17576,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496659726383</t>
         </is>
       </c>
+      <c r="O271" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cotton-jhola</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="3" t="n">
@@ -16313,6 +17639,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496659759151</t>
         </is>
       </c>
+      <c r="O272" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cushion-cover  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="3" t="n">
@@ -16371,6 +17702,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496659759151</t>
         </is>
       </c>
+      <c r="O273" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cushion-cover  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" s="3" t="n">
@@ -16429,6 +17765,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496659890223</t>
         </is>
       </c>
+      <c r="O274" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cotton-bedspread-king-1  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="3" t="n">
@@ -16487,6 +17828,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496659922991</t>
         </is>
       </c>
+      <c r="O275" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cotton-bedspread-king-2  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" s="3" t="n">
@@ -16545,6 +17891,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496659857455</t>
         </is>
       </c>
+      <c r="O276" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cotton-bedspread-king  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="3" t="n">
@@ -16603,6 +17954,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496659988527</t>
         </is>
       </c>
+      <c r="O277" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cotton-bed-spread-queen-1  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" s="3" t="n">
@@ -16661,6 +18017,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660021295</t>
         </is>
       </c>
+      <c r="O278" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cotton-bed-spread-queen-2  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="3" t="n">
@@ -16719,6 +18080,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496659955759</t>
         </is>
       </c>
+      <c r="O279" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cotton-bed-spread-queen  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="3" t="n">
@@ -16777,6 +18143,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660217903</t>
         </is>
       </c>
+      <c r="O280" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-bedspread-single-2  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="3" t="n">
@@ -16835,6 +18206,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660283439</t>
         </is>
       </c>
+      <c r="O281" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-bedspread-single-4  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="3" t="n">
@@ -16893,6 +18269,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660119599</t>
         </is>
       </c>
+      <c r="O282" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-bedspread-single-1  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="3" t="n">
@@ -16951,6 +18332,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660283439</t>
         </is>
       </c>
+      <c r="O283" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-bedspread-single-4  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="3" t="n">
@@ -17009,6 +18395,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660250671</t>
         </is>
       </c>
+      <c r="O284" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-bedspread-single-3  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="3" t="n">
@@ -17067,6 +18458,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660316207</t>
         </is>
       </c>
+      <c r="O285" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-bedspread-single-5  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="3" t="n">
@@ -17121,6 +18517,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660348975</t>
         </is>
       </c>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-wrapper</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="3" t="n">
@@ -17175,6 +18576,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660381743</t>
         </is>
       </c>
+      <c r="O287" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-wrapper-1</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="3" t="n">
@@ -17229,6 +18635,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660414511</t>
         </is>
       </c>
+      <c r="O288" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-wrapper-2</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="3" t="n">
@@ -17283,6 +18694,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660447279</t>
         </is>
       </c>
+      <c r="O289" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/assamese-wrapper</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="3" t="n">
@@ -17337,6 +18753,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660480047</t>
         </is>
       </c>
+      <c r="O290" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/naga-wrapper-3</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="3" t="n">
@@ -17391,6 +18812,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660545583</t>
         </is>
       </c>
+      <c r="O291" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/assamese-wrapper-2</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="3" t="n">
@@ -17453,6 +18879,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660578351</t>
         </is>
       </c>
+      <c r="O292" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/off-white-jamdani-lamp-with-wrought-iron-stand  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="3" t="n">
@@ -17515,6 +18946,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660611119</t>
         </is>
       </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madurkathi-table-mat-set-with-runner-6-1</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" s="3" t="n">
@@ -17577,6 +19013,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660611119</t>
         </is>
       </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madurkathi-table-mat-set-with-runner-6-1</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" s="3" t="n">
@@ -17643,6 +19084,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660611119</t>
         </is>
       </c>
+      <c r="O295" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madurkathi-table-mat-set-with-runner-6-1</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="3" t="n">
@@ -17710,6 +19156,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660611119</t>
         </is>
       </c>
+      <c r="O296" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madurkathi-table-mat-set-with-runner-6-1</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="3" t="n">
@@ -17772,6 +19223,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660611119</t>
         </is>
       </c>
+      <c r="O297" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/madurkathi-table-mat-set-with-runner-6-1</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="3" t="n">
@@ -17826,6 +19282,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660676655</t>
         </is>
       </c>
+      <c r="O298" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/uttoriyo-cushion-cover-16-by-16</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="3" t="n">
@@ -17880,6 +19341,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660742191</t>
         </is>
       </c>
+      <c r="O299" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-crafted-beads-waterfall-necklace</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="3" t="n">
@@ -17940,6 +19406,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660774959</t>
         </is>
       </c>
+      <c r="O300" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-u-bag  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="3" t="n">
@@ -18003,6 +19474,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660807727</t>
         </is>
       </c>
+      <c r="O301" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-bag  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" s="3" t="n">
@@ -18057,6 +19533,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660840495</t>
         </is>
       </c>
+      <c r="O302" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/round-hand-embroidered-place-mat</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" s="3" t="n">
@@ -18111,6 +19592,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660906031</t>
         </is>
       </c>
+      <c r="O303" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/rectangular-hand-embroidered-place-mat</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" s="3" t="n">
@@ -18165,6 +19651,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660938799</t>
         </is>
       </c>
+      <c r="O304" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/rectangular-hand-embroidered-place-mat-1</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="3" t="n">
@@ -18219,6 +19710,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496661102639</t>
         </is>
       </c>
+      <c r="O305" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/kauna-cherry-bag-with-bhoomija-logo  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="3" t="n">
@@ -18281,6 +19777,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496661135407</t>
         </is>
       </c>
+      <c r="O306" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroirdered-kauna-moon-clutch  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="3" t="n">
@@ -18343,6 +19844,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496661135407</t>
         </is>
       </c>
+      <c r="O307" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroirdered-kauna-moon-clutch  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="3" t="n">
@@ -18406,6 +19912,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496661200943</t>
         </is>
       </c>
+      <c r="O308" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/kauna-hamper-basket-rectangular</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="3" t="n">
@@ -18460,6 +19971,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496661266479</t>
         </is>
       </c>
+      <c r="O309" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/kauna-hamper-basket-oval</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="3" t="n">
@@ -18514,6 +20030,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496661364783</t>
         </is>
       </c>
+      <c r="O310" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/nagamese-hairpin</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" s="3" t="n">
@@ -18572,6 +20093,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496661430319</t>
         </is>
       </c>
+      <c r="O311" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/nagamese-konyak-traditional-open-necklace</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" s="3" t="n">
@@ -18630,6 +20156,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496661495855</t>
         </is>
       </c>
+      <c r="O312" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/nagamese-necklace</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" s="3" t="n">
@@ -18688,6 +20219,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496661463087</t>
         </is>
       </c>
+      <c r="O313" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/nagamese-net-necklace</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" s="3" t="n">
@@ -18740,6 +20276,11 @@
       <c r="N314" s="3" t="inlineStr">
         <is>
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496661561391</t>
+        </is>
+      </c>
+      <c r="O314" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/tikuli-hand-painted-mirror</t>
         </is>
       </c>
     </row>
@@ -18755,7 +20296,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -18764,6 +20305,7 @@
     <col width="25" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -18797,6 +20339,11 @@
           <t>Admin link</t>
         </is>
       </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Live product link</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -18829,6 +20376,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496618405935</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/ashtalakshmi-stole-eight-sisters-embroidered</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -18861,6 +20413,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496640196655</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/wooden-serviette-fish-shaped</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -18893,6 +20450,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496641835055</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sohrai-11-by-15  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -18925,6 +20487,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496641835055</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/sohrai-11-by-15  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -18957,6 +20524,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496646553647</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/handwoven-mekhala-chador-from-assam-2  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -18989,6 +20561,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496653140015</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/red-tikuli-hand-painted-tray</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -19021,6 +20598,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496658186287</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/hand-embroidered-sujani-cushion-cover-16-by-16  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -19053,6 +20635,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496659791919</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cushion-cover-1  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -19085,6 +20672,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496659791919</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cushion-cover-1  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -19117,6 +20709,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496659791919</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cushion-cover-1  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -19149,6 +20746,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496659791919</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cushion-cover-1  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -19181,6 +20783,11 @@
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496659791919</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/bawan-buti-cushion-cover-1  (draft – not visible)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -19211,6 +20818,11 @@
       <c r="F14" t="inlineStr">
         <is>
           <t>https://admin.shopify.com/store/bhoomija-2/products/8496660512815</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>https://bhoomija.in/products/assamese-wrapper-1</t>
         </is>
       </c>
     </row>

</xml_diff>